<commit_message>
Never claim an unlabeled column that holds data; match the real sheet's tab and column names
The Status column check now looks at every cell, not just the header, after
finding that the real Manual Entry tab has an unlabeled but filled column
right after Tracking. Practice data now mirrors the real sheet layout.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01YPdQ6TbQXaCbDqbgrqrFk1
</commit_message>
<xml_diff>
--- a/data/sample_tracking.xlsx
+++ b/data/sample_tracking.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet name="Form Responses 1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Manual Entries" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Manual Entry" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -417,51 +417,61 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:K7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>Date</t>
+          <t>Timestamp</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Name</t>
+          <t>Quantity of Santa Pants Cocktail "Garnishes" Requested (150 per order)</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Address</t>
+          <t>Account Name</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Address 2</t>
+          <t>Shipping Address</t>
         </is>
       </c>
       <c r="E1" t="inlineStr">
         <is>
-          <t>City</t>
+          <t>City &amp; State</t>
         </is>
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>State</t>
+          <t>Zip Code</t>
         </is>
       </c>
       <c r="G1" t="inlineStr">
         <is>
-          <t>ZIP code</t>
+          <t>Contact Phone Number</t>
         </is>
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Kit quantity</t>
+          <t>Email</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
+        <is>
+          <t>Preferred Delivery Window</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Account Instagram Handle (for Social Promotions)</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
         <is>
           <t>Tracking</t>
         </is>
@@ -471,33 +481,33 @@
       <c r="A2" s="1" t="n">
         <v>46301</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Avery Example</t>
-        </is>
+      <c r="B2" t="n">
+        <v>1</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Example Tavern</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>100 Sample St</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Columbus</t>
-        </is>
-      </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>OH</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
+          <t>Columbus, OH</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
         <v>43004</v>
       </c>
-      <c r="H2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I2" t="n">
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>Week of November 2 (first available)</t>
+        </is>
+      </c>
+      <c r="K2" t="n">
         <v>100000000001</v>
       </c>
     </row>
@@ -505,38 +515,38 @@
       <c r="A3" s="1" t="n">
         <v>46302</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Jordan Placeholder</t>
-        </is>
+      <c r="B3" t="n">
+        <v>2</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>22 Test Ave</t>
+          <t>Placeholder Lounge</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Suite 4</t>
+          <t>22 Test Ave Suite 4</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Denver</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>CO</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
+          <t>Denver, CO</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
         <v>80014</v>
       </c>
-      <c r="H3" t="n">
-        <v>1</v>
-      </c>
       <c r="I3" t="inlineStr">
+        <is>
+          <t>Week of November 2 (first available)</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>@placeholderlounge</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
         <is>
           <t>1000 0000 0003</t>
         </is>
@@ -546,33 +556,33 @@
       <c r="A4" s="1" t="n">
         <v>46303</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Riley Demo</t>
-        </is>
+      <c r="B4" t="n">
+        <v>1</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Demo Bar &amp; Grill</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>9 Mock Rd</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Austin</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>TX</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
+          <t>Austin, TX</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
         <v>73301</v>
       </c>
-      <c r="H4" t="n">
-        <v>3</v>
-      </c>
-      <c r="I4" t="n">
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>Week of November 2 (first available)</t>
+        </is>
+      </c>
+      <c r="K4" t="n">
         <v>100000000006</v>
       </c>
     </row>
@@ -580,33 +590,33 @@
       <c r="A5" s="1" t="n">
         <v>46304</v>
       </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Casey Fiction</t>
-        </is>
+      <c r="B5" t="n">
+        <v>1</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
+          <t>Fiction Pub</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
           <t>450 Fake Blvd</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Tampa</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>FL</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
+          <t>Tampa, FL</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
         <v>33601</v>
       </c>
-      <c r="H5" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" t="n">
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>Week of November 2 (first available)</t>
+        </is>
+      </c>
+      <c r="K5" t="n">
         <v>100000000007</v>
       </c>
     </row>
@@ -614,69 +624,64 @@
       <c r="A6" s="1" t="n">
         <v>46305</v>
       </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Morgan Sample</t>
-        </is>
+      <c r="B6" t="n">
+        <v>3</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>7 Pretend Ln</t>
+          <t>Sample Spirits Co</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Apt 2B</t>
+          <t>7 Pretend Ln Apt 2B</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Portland</t>
-        </is>
-      </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>OR</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
+          <t>Portland, OR</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
         <v>97035</v>
       </c>
-      <c r="H6" t="n">
-        <v>2</v>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>Week of November 2 (first available)</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
         <v>46305</v>
       </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>Quinn Invented</t>
-        </is>
+      <c r="B7" t="n">
+        <v>1</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
+          <t>Invented Inn</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
           <t>31 Imaginary Way</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Raleigh</t>
-        </is>
-      </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>NC</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
+          <t>Raleigh, NC</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
         <v>27601</v>
       </c>
-      <c r="H7" t="n">
-        <v>1</v>
-      </c>
       <c r="I7" t="inlineStr">
+        <is>
+          <t>Week of November 2 (first available)</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
         <is>
           <t>1.00000E+11</t>
         </is>
@@ -693,155 +698,171 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" t="inlineStr"/>
+      <c r="B1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>Address</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>Address 2</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>State</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>ZIP code</t>
-        </is>
-      </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Kit quantity</t>
+          <t>Zip Code</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
         <is>
+          <t>Kit Quantity</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
           <t>Tracking</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="n">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Holiday 26</t>
+        </is>
+      </c>
+      <c r="B2" s="1" t="n">
         <v>46300</v>
       </c>
-      <c r="B2" t="inlineStr">
-        <is>
-          <t>Taylor Madeup</t>
-        </is>
-      </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>Madeup Taproom</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>8 Nowhere Ct</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="F2" t="inlineStr">
         <is>
           <t>Boise</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="G2" t="inlineStr">
         <is>
           <t>ID</t>
         </is>
       </c>
-      <c r="G2" t="n">
+      <c r="H2" t="n">
         <v>83702</v>
       </c>
-      <c r="H2" t="n">
+      <c r="I2" t="n">
         <v>4</v>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>100000000002</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="1" t="n">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Holiday 26</t>
+        </is>
+      </c>
+      <c r="B3" s="1" t="n">
         <v>46304</v>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Drew Synthetic</t>
-        </is>
-      </c>
       <c r="C3" t="inlineStr">
         <is>
+          <t>Synthetic Saloon</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
           <t>64 Specimen Dr</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr">
+      <c r="F3" t="inlineStr">
         <is>
           <t>Omaha</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr">
+      <c r="G3" t="inlineStr">
         <is>
           <t>NE</t>
         </is>
       </c>
-      <c r="G3" t="n">
+      <c r="H3" t="n">
         <v>68102</v>
       </c>
-      <c r="H3" t="n">
+      <c r="I3" t="n">
         <v>1</v>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>100000000009</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="1" t="n">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Holiday 26</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="n">
         <v>46306</v>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Sam Notreal</t>
-        </is>
-      </c>
       <c r="C4" t="inlineStr">
         <is>
+          <t>Notreal Brewhouse</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
           <t>12 Hypothetical Pl</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="F4" t="inlineStr">
         <is>
           <t>Madison</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="G4" t="inlineStr">
         <is>
           <t>WI</t>
         </is>
       </c>
-      <c r="G4" t="n">
+      <c r="H4" t="n">
         <v>53703</v>
       </c>
-      <c r="H4" t="n">
+      <c r="I4" t="n">
         <v>2</v>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>999999999999</v>
       </c>
     </row>

</xml_diff>